<commit_message>
Update strategies and funding display
</commit_message>
<xml_diff>
--- a/data_raw/strategies.xlsx
+++ b/data_raw/strategies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/courtney/Desktop/ab617-dashboard/ab617-dashboard/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22108FAC-894B-DD44-B41B-1A5C1B798C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D566F56-09E5-1340-8978-787DBB87E838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full" sheetId="2" r:id="rId1"/>
@@ -4926,7 +4926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:W518"/>
@@ -5151,7 +5151,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="372" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" ht="356" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
@@ -5321,7 +5321,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:23" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>20</v>
       </c>
@@ -5367,7 +5367,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" ht="85" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>20</v>
       </c>
@@ -5413,7 +5413,7 @@
         <v>1119</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:23" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>20</v>
       </c>
@@ -5780,7 +5780,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="170" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:23" ht="153" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>98</v>
       </c>
@@ -5843,7 +5843,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="170" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:23" ht="153" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>98</v>
       </c>
@@ -6340,7 +6340,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
         <v>98</v>
       </c>
@@ -6901,7 +6901,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="108.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:23" ht="108.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
         <v>98</v>
       </c>
@@ -6962,7 +6962,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
         <v>20</v>
       </c>
@@ -7071,7 +7071,7 @@
         <v>1243</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
         <v>20</v>
       </c>
@@ -7195,7 +7195,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="92.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:23" ht="92.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="6" t="s">
         <v>98</v>
       </c>
@@ -7263,7 +7263,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="6" t="s">
         <v>32</v>
       </c>
@@ -7323,7 +7323,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="6" t="s">
         <v>233</v>
       </c>
@@ -7452,7 +7452,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
         <v>20</v>
       </c>
@@ -7723,7 +7723,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>58</v>
       </c>
@@ -7792,7 +7792,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>132</v>
       </c>
@@ -8046,7 +8046,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="67.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:23" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
         <v>20</v>
       </c>
@@ -8116,7 +8116,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
         <v>58</v>
       </c>
@@ -8185,7 +8185,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="6" t="s">
         <v>32</v>
       </c>
@@ -8244,7 +8244,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
         <v>233</v>
       </c>
@@ -8375,7 +8375,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
         <v>20</v>
       </c>
@@ -8434,7 +8434,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
         <v>98</v>
       </c>
@@ -8573,7 +8573,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
         <v>2</v>
       </c>
@@ -8852,7 +8852,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="6" t="s">
         <v>205</v>
       </c>
@@ -8913,7 +8913,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="6" t="s">
         <v>2</v>
       </c>
@@ -8967,7 +8967,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="65" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
         <v>205</v>
       </c>
@@ -9026,7 +9026,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
         <v>205</v>
       </c>
@@ -9091,7 +9091,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
         <v>233</v>
       </c>
@@ -9152,7 +9152,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
         <v>233</v>
       </c>
@@ -9213,7 +9213,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
         <v>32</v>
       </c>
@@ -9272,7 +9272,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
         <v>98</v>
       </c>
@@ -9331,7 +9331,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
         <v>205</v>
       </c>
@@ -9388,7 +9388,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
         <v>205</v>
       </c>
@@ -9438,7 +9438,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="71.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:23" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="8" t="s">
         <v>205</v>
       </c>
@@ -9494,7 +9494,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
         <v>20</v>
       </c>
@@ -9555,7 +9555,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="76.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:23" ht="76.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
         <v>20</v>
       </c>
@@ -9616,7 +9616,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
         <v>32</v>
       </c>
@@ -9681,7 +9681,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="77" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="6" t="s">
         <v>233</v>
       </c>
@@ -9742,7 +9742,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="6" t="s">
         <v>98</v>
       </c>
@@ -9803,7 +9803,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="6" t="s">
         <v>98</v>
       </c>
@@ -9862,7 +9862,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="6" t="s">
         <v>98</v>
       </c>
@@ -9923,7 +9923,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="81" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="6" t="s">
         <v>32</v>
       </c>
@@ -9984,7 +9984,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="82" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="6" t="s">
         <v>32</v>
       </c>
@@ -10045,7 +10045,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="83" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="6" t="s">
         <v>32</v>
       </c>
@@ -10106,7 +10106,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="6" t="s">
         <v>32</v>
       </c>
@@ -10167,7 +10167,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="85" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="6" t="s">
         <v>32</v>
       </c>
@@ -10228,7 +10228,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="6" t="s">
         <v>32</v>
       </c>
@@ -10289,7 +10289,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="87" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="6" t="s">
         <v>233</v>
       </c>
@@ -10350,7 +10350,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="6" t="s">
         <v>32</v>
       </c>
@@ -10411,7 +10411,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="84.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:23" ht="84.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="6" t="s">
         <v>205</v>
       </c>
@@ -10472,7 +10472,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="90" spans="1:23" ht="125.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:23" ht="125.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="6" t="s">
         <v>205</v>
       </c>
@@ -10533,7 +10533,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="91" spans="1:23" ht="114.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:23" ht="114.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="6" t="s">
         <v>205</v>
       </c>
@@ -10594,7 +10594,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="92" spans="1:23" ht="103.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:23" ht="103.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="6" t="s">
         <v>32</v>
       </c>
@@ -10655,7 +10655,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="93" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="6" t="s">
         <v>58</v>
       </c>
@@ -10714,7 +10714,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="6" t="s">
         <v>205</v>
       </c>
@@ -10775,7 +10775,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="147" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:23" ht="147" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="6" t="s">
         <v>205</v>
       </c>
@@ -10836,7 +10836,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="109.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:23" ht="109.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="6" t="s">
         <v>205</v>
       </c>
@@ -10897,7 +10897,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="6" t="s">
         <v>205</v>
       </c>
@@ -10958,7 +10958,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="6" t="s">
         <v>32</v>
       </c>
@@ -11019,7 +11019,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="6" t="s">
         <v>32</v>
       </c>
@@ -11080,7 +11080,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="6" t="s">
         <v>98</v>
       </c>
@@ -11141,7 +11141,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="6" t="s">
         <v>58</v>
       </c>
@@ -11200,7 +11200,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="6" t="s">
         <v>205</v>
       </c>
@@ -11261,7 +11261,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="62.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:23" ht="62.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="6" t="s">
         <v>205</v>
       </c>
@@ -11320,7 +11320,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="6" t="s">
         <v>233</v>
       </c>
@@ -11381,7 +11381,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="6" t="s">
         <v>233</v>
       </c>
@@ -11442,7 +11442,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="6" t="s">
         <v>233</v>
       </c>
@@ -11503,7 +11503,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="107" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="6" t="s">
         <v>233</v>
       </c>
@@ -11564,7 +11564,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="6" t="s">
         <v>58</v>
       </c>
@@ -11623,7 +11623,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="6" t="s">
         <v>98</v>
       </c>
@@ -11684,7 +11684,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="6" t="s">
         <v>32</v>
       </c>
@@ -11745,7 +11745,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="111" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="6" t="s">
         <v>98</v>
       </c>
@@ -11799,7 +11799,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="112" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="6" t="s">
         <v>98</v>
       </c>
@@ -11853,7 +11853,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="113" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="6" t="s">
         <v>32</v>
       </c>
@@ -11914,7 +11914,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="114" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="6" t="s">
         <v>32</v>
       </c>
@@ -11974,7 +11974,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="115" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="6" t="s">
         <v>58</v>
       </c>
@@ -12035,7 +12035,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="6" t="s">
         <v>98</v>
       </c>
@@ -12096,7 +12096,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="117" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="6" t="s">
         <v>205</v>
       </c>
@@ -12157,7 +12157,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="118" spans="1:23" ht="55.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:23" ht="55.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="6" t="s">
         <v>20</v>
       </c>
@@ -12216,7 +12216,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="119" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="6" t="s">
         <v>205</v>
       </c>
@@ -12272,7 +12272,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="120" spans="1:23" ht="53.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:23" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="6" t="s">
         <v>98</v>
       </c>
@@ -12333,7 +12333,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="6" t="s">
         <v>205</v>
       </c>
@@ -12392,7 +12392,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="122" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="6" t="s">
         <v>32</v>
       </c>
@@ -12453,7 +12453,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="123" spans="1:23" ht="68.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:23" ht="68.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="6" t="s">
         <v>32</v>
       </c>
@@ -12512,7 +12512,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="124" spans="1:23" ht="128.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:23" ht="128.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="6" t="s">
         <v>233</v>
       </c>
@@ -12573,7 +12573,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="131.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:23" ht="131.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="6" t="s">
         <v>98</v>
       </c>
@@ -12631,7 +12631,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="126" spans="1:23" ht="66" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:23" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="6" t="s">
         <v>205</v>
       </c>
@@ -12689,7 +12689,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="127" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="6" t="s">
         <v>205</v>
       </c>
@@ -12747,7 +12747,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="6" t="s">
         <v>98</v>
       </c>
@@ -12805,7 +12805,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="6" t="s">
         <v>32</v>
       </c>
@@ -12865,7 +12865,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="130" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="6" t="s">
         <v>20</v>
       </c>
@@ -12931,7 +12931,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="131" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="6" t="s">
         <v>98</v>
       </c>
@@ -12986,7 +12986,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="132" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="6" t="s">
         <v>98</v>
       </c>
@@ -13041,7 +13041,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="133" spans="1:23" ht="85.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:23" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="6" t="s">
         <v>98</v>
       </c>
@@ -13096,7 +13096,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="134" spans="1:23" ht="176.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:23" ht="176.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="6" t="s">
         <v>98</v>
       </c>
@@ -13151,7 +13151,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="135" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="6" t="s">
         <v>98</v>
       </c>
@@ -13211,7 +13211,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="6" t="s">
         <v>58</v>
       </c>
@@ -13268,7 +13268,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="137" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="6" t="s">
         <v>58</v>
       </c>
@@ -13325,7 +13325,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="138" spans="1:23" ht="53.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:23" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="6" t="s">
         <v>20</v>
       </c>
@@ -13385,7 +13385,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="139" spans="1:23" ht="58.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:23" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="6" t="s">
         <v>20</v>
       </c>
@@ -13445,7 +13445,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="6" t="s">
         <v>32</v>
       </c>
@@ -13503,7 +13503,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="6" t="s">
         <v>58</v>
       </c>
@@ -13557,7 +13557,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="142" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="6" t="s">
         <v>132</v>
       </c>
@@ -13611,7 +13611,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="6" t="s">
         <v>132</v>
       </c>
@@ -13665,7 +13665,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="6" t="s">
         <v>132</v>
       </c>
@@ -13720,7 +13720,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="6" t="s">
         <v>132</v>
       </c>
@@ -13775,7 +13775,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="146" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="6" t="s">
         <v>132</v>
       </c>
@@ -13829,7 +13829,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="147" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="6" t="s">
         <v>172</v>
       </c>
@@ -13886,7 +13886,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="6" t="s">
         <v>172</v>
       </c>
@@ -13943,7 +13943,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="149" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="6" t="s">
         <v>32</v>
       </c>
@@ -14002,7 +14002,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="6" t="s">
         <v>32</v>
       </c>
@@ -14059,7 +14059,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="6" t="s">
         <v>205</v>
       </c>
@@ -14118,7 +14118,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="6" t="s">
         <v>205</v>
       </c>
@@ -14177,7 +14177,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="153" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="6" t="s">
         <v>205</v>
       </c>
@@ -14236,7 +14236,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="154" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="6" t="s">
         <v>205</v>
       </c>
@@ -14293,7 +14293,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="155" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="6" t="s">
         <v>98</v>
       </c>
@@ -14350,7 +14350,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="6" t="s">
         <v>205</v>
       </c>
@@ -14409,7 +14409,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="6" t="s">
         <v>205</v>
       </c>
@@ -14466,7 +14466,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="6" t="s">
         <v>32</v>
       </c>
@@ -14525,7 +14525,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="159" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="6" t="s">
         <v>172</v>
       </c>
@@ -14581,7 +14581,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="97.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:23" ht="97.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="6" t="s">
         <v>172</v>
       </c>
@@ -14853,7 +14853,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="6" t="s">
         <v>205</v>
       </c>
@@ -14916,7 +14916,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="6" t="s">
         <v>205</v>
       </c>
@@ -14979,7 +14979,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="166" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="6" t="s">
         <v>32</v>
       </c>
@@ -15046,7 +15046,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="167" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="6" t="s">
         <v>233</v>
       </c>
@@ -15177,7 +15177,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="169" spans="1:23" ht="103.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:23" ht="103.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="6" t="s">
         <v>58</v>
       </c>
@@ -15247,7 +15247,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="6" t="s">
         <v>172</v>
       </c>
@@ -15315,7 +15315,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="171" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="6" t="s">
         <v>205</v>
       </c>
@@ -15381,7 +15381,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="172" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="6" t="s">
         <v>205</v>
       </c>
@@ -15505,7 +15505,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="6" t="s">
         <v>205</v>
       </c>
@@ -15581,7 +15581,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="6" t="s">
         <v>32</v>
       </c>
@@ -15645,7 +15645,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="9" t="s">
         <v>172</v>
       </c>
@@ -15697,7 +15697,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="177" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="8" t="s">
         <v>172</v>
       </c>
@@ -15749,7 +15749,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="178" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="8" t="s">
         <v>172</v>
       </c>
@@ -15801,7 +15801,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="6" t="s">
         <v>205</v>
       </c>
@@ -15859,7 +15859,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="6" t="s">
         <v>98</v>
       </c>
@@ -15916,7 +15916,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="181" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="6" t="s">
         <v>205</v>
       </c>
@@ -15964,7 +15964,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="182" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="6" t="s">
         <v>205</v>
       </c>
@@ -16012,7 +16012,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="6" t="s">
         <v>58</v>
       </c>
@@ -16132,7 +16132,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="6" t="s">
         <v>205</v>
       </c>
@@ -16193,7 +16193,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="186" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="6" t="s">
         <v>32</v>
       </c>
@@ -16254,7 +16254,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="187" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="6" t="s">
         <v>98</v>
       </c>
@@ -16313,7 +16313,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="188" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="6" t="s">
         <v>98</v>
       </c>
@@ -16372,7 +16372,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="189" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="6" t="s">
         <v>205</v>
       </c>
@@ -16429,7 +16429,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="6" t="s">
         <v>205</v>
       </c>
@@ -16486,7 +16486,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="191" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="6" t="s">
         <v>205</v>
       </c>
@@ -16545,7 +16545,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" s="6" t="s">
         <v>58</v>
       </c>
@@ -16606,7 +16606,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="193" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="6" t="s">
         <v>205</v>
       </c>
@@ -16665,7 +16665,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="194" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="6" t="s">
         <v>205</v>
       </c>
@@ -16730,7 +16730,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="195" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="6" t="s">
         <v>205</v>
       </c>
@@ -16787,7 +16787,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="196" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" s="8" t="s">
         <v>205</v>
       </c>
@@ -16839,7 +16839,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="197" spans="1:23" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:23" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197" s="6" t="s">
         <v>32</v>
       </c>
@@ -16896,7 +16896,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="198" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198" s="6" t="s">
         <v>205</v>
       </c>
@@ -16955,7 +16955,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="199" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199" s="6" t="s">
         <v>205</v>
       </c>
@@ -17014,7 +17014,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="200" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A200" s="6" t="s">
         <v>205</v>
       </c>
@@ -17073,7 +17073,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="201" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201" s="6" t="s">
         <v>32</v>
       </c>
@@ -17132,7 +17132,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="202" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A202" s="6" t="s">
         <v>20</v>
       </c>
@@ -17184,7 +17184,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="203" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A203" s="6" t="s">
         <v>20</v>
       </c>
@@ -17236,7 +17236,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="204" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A204" s="6" t="s">
         <v>32</v>
       </c>
@@ -17293,7 +17293,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="205" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205" s="6" t="s">
         <v>58</v>
       </c>
@@ -17345,7 +17345,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="206" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A206" s="6" t="s">
         <v>58</v>
       </c>
@@ -17397,7 +17397,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="207" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A207" s="6" t="s">
         <v>132</v>
       </c>
@@ -17449,7 +17449,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="208" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A208" s="6" t="s">
         <v>205</v>
       </c>
@@ -17506,7 +17506,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="209" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209" s="6" t="s">
         <v>132</v>
       </c>
@@ -17558,7 +17558,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="210" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A210" s="6" t="s">
         <v>205</v>
       </c>
@@ -17668,7 +17668,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="212" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A212" s="6" t="s">
         <v>205</v>
       </c>
@@ -17726,7 +17726,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="213" spans="1:23" ht="50.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:23" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A213" s="6" t="s">
         <v>205</v>
       </c>
@@ -17782,7 +17782,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="214" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="6" t="s">
         <v>205</v>
       </c>
@@ -17830,7 +17830,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="215" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="6" t="s">
         <v>205</v>
       </c>
@@ -17878,7 +17878,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="216" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="6" t="s">
         <v>205</v>
       </c>
@@ -17926,7 +17926,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="217" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="6" t="s">
         <v>205</v>
       </c>
@@ -17974,7 +17974,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="218" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A218" s="6" t="s">
         <v>205</v>
       </c>
@@ -18022,7 +18022,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="219" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219" s="8" t="s">
         <v>205</v>
       </c>
@@ -18072,7 +18072,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="220" spans="1:23" ht="95.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:23" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A220" s="6" t="s">
         <v>205</v>
       </c>
@@ -18120,7 +18120,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="221" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A221" s="6" t="s">
         <v>205</v>
       </c>
@@ -18168,7 +18168,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="222" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A222" s="6" t="s">
         <v>205</v>
       </c>
@@ -18216,7 +18216,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="223" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A223" s="6" t="s">
         <v>205</v>
       </c>
@@ -18264,7 +18264,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="224" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A224" s="6" t="s">
         <v>205</v>
       </c>
@@ -18320,7 +18320,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="225" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A225" s="6" t="s">
         <v>205</v>
       </c>
@@ -18376,7 +18376,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="226" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A226" s="6" t="s">
         <v>205</v>
       </c>
@@ -18432,7 +18432,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="227" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A227" s="6" t="s">
         <v>205</v>
       </c>
@@ -18488,7 +18488,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="228" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A228" s="6" t="s">
         <v>205</v>
       </c>
@@ -18544,7 +18544,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="229" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A229" s="6" t="s">
         <v>205</v>
       </c>
@@ -18600,7 +18600,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="230" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A230" s="6" t="s">
         <v>205</v>
       </c>
@@ -18656,7 +18656,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="231" spans="1:23" ht="77.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:23" ht="77.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A231" s="6" t="s">
         <v>205</v>
       </c>
@@ -18712,7 +18712,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="232" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A232" s="6" t="s">
         <v>205</v>
       </c>
@@ -18762,7 +18762,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="233" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A233" s="6" t="s">
         <v>205</v>
       </c>
@@ -18810,7 +18810,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="234" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A234" s="6" t="s">
         <v>205</v>
       </c>
@@ -18858,7 +18858,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="235" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A235" s="6" t="s">
         <v>205</v>
       </c>
@@ -18906,7 +18906,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="236" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A236" s="6" t="s">
         <v>205</v>
       </c>
@@ -18956,7 +18956,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="237" spans="1:23" ht="78.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:23" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A237" s="6" t="s">
         <v>205</v>
       </c>
@@ -19006,7 +19006,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="238" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A238" s="6" t="s">
         <v>205</v>
       </c>
@@ -19054,7 +19054,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="239" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A239" s="6" t="s">
         <v>20</v>
       </c>
@@ -19102,7 +19102,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="240" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A240" s="6" t="s">
         <v>20</v>
       </c>
@@ -19150,7 +19150,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="241" spans="1:23" ht="129.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:23" ht="129.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A241" s="6" t="s">
         <v>20</v>
       </c>
@@ -19200,7 +19200,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="242" spans="1:23" ht="76.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:23" ht="76.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A242" s="6" t="s">
         <v>20</v>
       </c>
@@ -19250,7 +19250,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="243" spans="1:23" ht="63.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:23" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A243" s="6" t="s">
         <v>20</v>
       </c>
@@ -19300,7 +19300,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="244" spans="1:23" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:23" ht="83.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A244" s="6" t="s">
         <v>20</v>
       </c>
@@ -19351,7 +19351,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="245" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A245" s="6" t="s">
         <v>205</v>
       </c>
@@ -19405,7 +19405,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="246" spans="1:23" ht="68.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:23" ht="68.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A246" s="6" t="s">
         <v>32</v>
       </c>
@@ -19464,7 +19464,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="247" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A247" s="6" t="s">
         <v>32</v>
       </c>
@@ -19514,7 +19514,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="248" spans="1:23" ht="62.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:23" ht="62.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A248" s="6" t="s">
         <v>32</v>
       </c>
@@ -19564,7 +19564,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="249" spans="1:23" ht="143.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:23" ht="143.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A249" s="6" t="s">
         <v>32</v>
       </c>
@@ -19612,7 +19612,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="250" spans="1:23" ht="57" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:23" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A250" s="6" t="s">
         <v>32</v>
       </c>
@@ -19660,7 +19660,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="251" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A251" s="6" t="s">
         <v>32</v>
       </c>
@@ -19708,7 +19708,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="252" spans="1:23" ht="87" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:23" ht="87" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A252" s="6" t="s">
         <v>233</v>
       </c>
@@ -19756,7 +19756,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="253" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A253" s="6" t="s">
         <v>233</v>
       </c>
@@ -19804,7 +19804,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="254" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A254" s="6" t="s">
         <v>233</v>
       </c>
@@ -19852,7 +19852,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="255" spans="1:23" ht="50.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:23" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A255" s="6" t="s">
         <v>233</v>
       </c>
@@ -19900,7 +19900,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="256" spans="1:23" ht="66.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:23" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256" s="6" t="s">
         <v>233</v>
       </c>
@@ -19948,7 +19948,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="257" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A257" s="6" t="s">
         <v>233</v>
       </c>
@@ -19996,7 +19996,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="258" spans="1:23" ht="39" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:23" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258" s="6" t="s">
         <v>233</v>
       </c>
@@ -20052,7 +20052,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="259" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A259" s="6" t="s">
         <v>233</v>
       </c>
@@ -20102,7 +20102,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="260" spans="1:23" ht="53.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:23" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="6" t="s">
         <v>233</v>
       </c>
@@ -20152,7 +20152,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="261" spans="1:23" ht="69" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:23" ht="69" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261" s="6" t="s">
         <v>233</v>
       </c>
@@ -20200,7 +20200,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="262" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A262" s="6" t="s">
         <v>233</v>
       </c>
@@ -20250,7 +20250,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="263" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263" s="6" t="s">
         <v>233</v>
       </c>
@@ -20298,7 +20298,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="264" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="6" t="s">
         <v>233</v>
       </c>
@@ -20348,7 +20348,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="265" spans="1:23" ht="46.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:23" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A265" s="6" t="s">
         <v>233</v>
       </c>
@@ -20396,7 +20396,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="266" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A266" s="6" t="s">
         <v>233</v>
       </c>
@@ -20444,7 +20444,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="267" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A267" s="6" t="s">
         <v>98</v>
       </c>
@@ -20492,7 +20492,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="268" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A268" s="6" t="s">
         <v>98</v>
       </c>
@@ -20542,7 +20542,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="269" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269" s="6" t="s">
         <v>98</v>
       </c>
@@ -20592,7 +20592,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="270" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A270" s="6" t="s">
         <v>98</v>
       </c>
@@ -20638,7 +20638,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="271" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A271" s="6" t="s">
         <v>98</v>
       </c>
@@ -20684,7 +20684,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="272" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A272" s="6" t="s">
         <v>98</v>
       </c>
@@ -20730,7 +20730,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="273" spans="1:23" ht="70.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:23" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A273" s="6" t="s">
         <v>98</v>
       </c>
@@ -20780,7 +20780,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="274" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A274" s="6" t="s">
         <v>98</v>
       </c>
@@ -20826,7 +20826,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="275" spans="1:23" ht="56.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:23" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A275" s="6" t="s">
         <v>98</v>
       </c>
@@ -20872,7 +20872,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="276" spans="1:23" ht="50.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:23" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A276" s="6" t="s">
         <v>98</v>
       </c>
@@ -20918,7 +20918,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="277" spans="1:23" ht="61.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:23" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A277" s="6" t="s">
         <v>2</v>
       </c>
@@ -20966,7 +20966,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="278" spans="1:23" ht="72" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:23" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A278" s="6" t="s">
         <v>2</v>
       </c>
@@ -21014,7 +21014,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="279" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A279" s="6" t="s">
         <v>2</v>
       </c>
@@ -21065,7 +21065,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="280" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A280" s="6" t="s">
         <v>2</v>
       </c>
@@ -21116,7 +21116,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="281" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A281" s="6" t="s">
         <v>2</v>
       </c>
@@ -21166,7 +21166,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="282" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A282" s="6" t="s">
         <v>2</v>
       </c>
@@ -21216,7 +21216,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="283" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A283" s="6" t="s">
         <v>2</v>
       </c>
@@ -21267,7 +21267,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="284" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A284" s="6" t="s">
         <v>2</v>
       </c>
@@ -21317,7 +21317,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="285" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A285" s="6" t="s">
         <v>58</v>
       </c>
@@ -21367,7 +21367,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="286" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A286" s="6" t="s">
         <v>58</v>
       </c>
@@ -21419,7 +21419,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="287" spans="1:23" ht="75.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:23" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A287" s="6" t="s">
         <v>58</v>
       </c>
@@ -21471,7 +21471,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="288" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A288" s="6" t="s">
         <v>58</v>
       </c>
@@ -21521,7 +21521,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="289" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A289" s="6" t="s">
         <v>58</v>
       </c>
@@ -21572,7 +21572,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="290" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A290" s="6" t="s">
         <v>58</v>
       </c>
@@ -21622,7 +21622,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="291" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A291" s="6" t="s">
         <v>58</v>
       </c>
@@ -21670,7 +21670,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="292" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A292" s="6" t="s">
         <v>58</v>
       </c>
@@ -21718,7 +21718,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="293" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A293" s="6" t="s">
         <v>58</v>
       </c>
@@ -21766,7 +21766,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="294" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A294" s="6" t="s">
         <v>58</v>
       </c>
@@ -21816,7 +21816,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="295" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A295" s="6" t="s">
         <v>132</v>
       </c>
@@ -21864,7 +21864,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="296" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A296" s="6" t="s">
         <v>132</v>
       </c>
@@ -21912,7 +21912,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="297" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A297" s="6" t="s">
         <v>132</v>
       </c>
@@ -21960,7 +21960,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="298" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A298" s="6" t="s">
         <v>132</v>
       </c>
@@ -22008,7 +22008,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="299" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A299" s="6" t="s">
         <v>132</v>
       </c>
@@ -22058,7 +22058,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="300" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A300" s="6" t="s">
         <v>132</v>
       </c>
@@ -22108,7 +22108,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="301" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A301" s="6" t="s">
         <v>132</v>
       </c>
@@ -22158,7 +22158,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="302" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A302" s="6" t="s">
         <v>132</v>
       </c>
@@ -22209,7 +22209,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="303" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A303" s="6" t="s">
         <v>132</v>
       </c>
@@ -22259,7 +22259,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="304" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A304" s="6" t="s">
         <v>132</v>
       </c>
@@ -22309,7 +22309,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="305" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A305" s="6" t="s">
         <v>172</v>
       </c>
@@ -22357,7 +22357,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="306" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A306" s="6" t="s">
         <v>172</v>
       </c>
@@ -22405,7 +22405,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="307" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A307" s="6" t="s">
         <v>172</v>
       </c>
@@ -22453,7 +22453,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="308" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A308" s="6" t="s">
         <v>172</v>
       </c>
@@ -22503,7 +22503,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="309" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A309" s="6" t="s">
         <v>172</v>
       </c>
@@ -22554,7 +22554,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="310" spans="1:23" ht="62.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:23" ht="62.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A310" s="6" t="s">
         <v>172</v>
       </c>
@@ -22604,7 +22604,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="311" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A311" s="6" t="s">
         <v>172</v>
       </c>
@@ -22652,7 +22652,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="312" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A312" s="6" t="s">
         <v>32</v>
       </c>
@@ -22711,7 +22711,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="313" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A313" s="6" t="s">
         <v>32</v>
       </c>
@@ -22770,7 +22770,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="314" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A314" s="6" t="s">
         <v>32</v>
       </c>
@@ -22829,7 +22829,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="315" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A315" s="6" t="s">
         <v>32</v>
       </c>
@@ -22888,7 +22888,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="316" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A316" s="6" t="s">
         <v>32</v>
       </c>
@@ -22947,7 +22947,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="317" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A317" s="6" t="s">
         <v>98</v>
       </c>
@@ -24105,7 +24105,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="336" spans="1:23" ht="131.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:23" ht="131.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A336" s="6" t="s">
         <v>58</v>
       </c>
@@ -24170,7 +24170,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="337" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A337" s="6" t="s">
         <v>205</v>
       </c>
@@ -24231,7 +24231,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="338" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A338" s="6" t="s">
         <v>233</v>
       </c>
@@ -24554,7 +24554,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="343" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A343" s="6" t="s">
         <v>205</v>
       </c>
@@ -24752,7 +24752,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="346" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A346" s="6" t="s">
         <v>205</v>
       </c>
@@ -24818,7 +24818,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="347" spans="1:23" ht="89.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:23" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A347" s="6" t="s">
         <v>205</v>
       </c>
@@ -24884,7 +24884,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="348" spans="1:23" ht="78.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:23" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A348" s="6" t="s">
         <v>2</v>
       </c>
@@ -25135,7 +25135,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="352" spans="1:23" ht="69.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:23" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A352" s="6" t="s">
         <v>205</v>
       </c>
@@ -25183,7 +25183,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="353" spans="1:23" ht="69.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:23" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A353" s="6" t="s">
         <v>205</v>
       </c>
@@ -26918,7 +26918,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="381" spans="1:23" ht="72" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="381" spans="1:23" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A381" s="6" t="s">
         <v>2</v>
       </c>
@@ -26989,7 +26989,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="382" spans="1:23" ht="72" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="382" spans="1:23" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A382" s="6" t="s">
         <v>132</v>
       </c>
@@ -28153,7 +28153,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="399" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="399" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A399" s="6" t="s">
         <v>58</v>
       </c>
@@ -28214,7 +28214,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="400" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="400" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A400" s="6" t="s">
         <v>132</v>
       </c>
@@ -28975,7 +28975,7 @@
         <v>100000</v>
       </c>
       <c r="O411" s="7">
-        <f t="shared" ref="O411:O442" si="24">M411+N411</f>
+        <f t="shared" ref="O411:O433" si="24">M411+N411</f>
         <v>486627.1</v>
       </c>
       <c r="P411" s="6">
@@ -30050,7 +30050,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="428" spans="1:23" ht="75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="428" spans="1:23" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A428" s="6" t="s">
         <v>58</v>
       </c>
@@ -30236,7 +30236,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="431" spans="1:23" ht="81" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="431" spans="1:23" ht="81" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A431" s="6" t="s">
         <v>58</v>
       </c>
@@ -30296,7 +30296,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="432" spans="1:23" ht="81" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="432" spans="1:23" ht="81" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A432" s="6" t="s">
         <v>132</v>
       </c>
@@ -30360,7 +30360,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="433" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="433" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A433" s="6" t="s">
         <v>172</v>
       </c>
@@ -30784,7 +30784,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="441" spans="1:23" ht="65.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="441" spans="1:23" ht="65.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A441" s="6" t="s">
         <v>132</v>
       </c>
@@ -31036,7 +31036,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="445" spans="1:23" ht="88.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="445" spans="1:23" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A445" s="6" t="s">
         <v>58</v>
       </c>
@@ -31915,7 +31915,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="459" spans="1:23" ht="54" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="459" spans="1:23" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A459" s="6" t="s">
         <v>132</v>
       </c>
@@ -32053,7 +32053,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="461" spans="1:23" ht="72.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="461" spans="1:23" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A461" s="6" t="s">
         <v>58</v>
       </c>
@@ -32118,7 +32118,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="462" spans="1:23" ht="81.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="462" spans="1:23" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A462" s="6" t="s">
         <v>172</v>
       </c>
@@ -32627,7 +32627,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="470" spans="1:23" ht="59.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="470" spans="1:23" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A470" s="6" t="s">
         <v>132</v>
       </c>
@@ -32696,7 +32696,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="471" spans="1:23" ht="64.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="471" spans="1:23" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A471" s="6" t="s">
         <v>2</v>
       </c>
@@ -32765,7 +32765,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="472" spans="1:23" ht="46.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="472" spans="1:23" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A472" s="6" t="s">
         <v>58</v>
       </c>
@@ -32834,7 +32834,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="473" spans="1:23" ht="66.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="473" spans="1:23" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A473" s="6" t="s">
         <v>172</v>
       </c>
@@ -33353,7 +33353,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="481" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="481" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A481" s="6" t="s">
         <v>58</v>
       </c>
@@ -34461,7 +34461,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="499" spans="1:23" ht="72.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="499" spans="1:23" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A499" s="6" t="s">
         <v>58</v>
       </c>
@@ -34780,7 +34780,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="504" spans="1:23" ht="80.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="504" spans="1:23" ht="80.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A504" s="8" t="s">
         <v>205</v>
       </c>
@@ -35650,7 +35650,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="518" spans="1:23" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="518" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A518" s="6" t="s">
         <v>205</v>
       </c>
@@ -35708,13 +35708,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W518" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="21">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:W518" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="R2:R396 R398:R518" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"School Districts,CalTrans,City,County,Air District,Community Centers (libraries,senior centers +),Industry - Port,Industry - Agriculture,Industry - Small Businesses,Industry,California Office of Environmental Health Hazard Assessment,CARB,San Diego Associ"&amp;"ation of Governance,CHP,Local Utilities &amp; Transportation,Public Health Agency,DPR"</formula1>

</xml_diff>